<commit_message>
docs: 기획서와 README 에 v0.4.0 ~ v0.4.7 변경 반영
- 기획서: 새 카드 11종 행 추가, 등급·확률·피해 단위·보스 체력 수치 갱신, 중첩 규칙 추가
- 기획서: '스테이지 구성' 시트(결투장 웨이브, 정예 스킬, 점프 버섯, 보물상자, 검증 봇 규칙) 추가
- 기획서: 상점 뽑기 가격 규칙과 카드 강화 가격·조작 정리
- README: 조작표(Tab, R), 카드 수와 버전 기록 갱신
</commit_message>
<xml_diff>
--- a/docs/design/roguelike_cards.xlsx
+++ b/docs/design/roguelike_cards.xlsx
@@ -15,10 +15,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경험치" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상점" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="캐릭터 패널" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보스 패턴" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스테이지 구성" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보스 패턴" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'카드 목록'!$A$1:$N$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'카드 목록'!$A$1:$N$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -816,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="22" customWidth="1" style="37" min="1" max="1"/>
@@ -986,12 +987,465 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="46" customHeight="1" s="37">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>능력치 창 (0.4.0)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>플레이 중 Tab 을 누르면 게임이 멈추고 능력치 창이 열린다. 왼쪽은 캐릭터 패널, 오른쪽은 얻은 카드 격자(능력치 카드 포함). 카드에 마우스를 올리거나 방향키로 고르면 아래에 등급·분류·단계와 수치가 들어간 자세한 설명이 나온다. Tab 이나 Esc 로 닫는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1" s="37">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>스테이지 1·2 개편 (0.4.0)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>매복 결투장, 점프 버섯, 정예 적, 보물상자를 넣어 단조롭던 구간을 나눈다. 자세한 배치는 '스테이지 구성' 시트.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1" s="37">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>0.4.1 변경</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>섀도우볼이 공격력 단계마다 바로 커지게 (그림 크기 = 반지름 x 2.3). 보스 체력 900. 보스 소환 박쥐는 플레이어를 향해 천천히 날아온다. 새 적 그림자 두꺼비, 정예 특별 스킬, 결투장 제한 시간·증원·붉은 경고 ('스테이지 구성' 시트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1" s="37">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>0.4.2 변경</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>피해를 10 단위로 (플레이어 기본 10, 공격력 +3/단계, 적 체력: 슬라임·마법사·두꺼비 20, 늑대 30, 박쥐 10, 스테이지마다 +10, 보스 3000). 새 카드 10종(혈사포, 레이저, 부메랑, 웨이브, 산탄, 무거운 공, 독, 냉기, 연쇄 번개, 그림자 궤도)과 등급 조정(유도·차지샷 전설-&gt;영웅, 튕김·저주 영웅-&gt;희귀). 카드로 겉모습이 바뀜(혈사포 뿔, 공중 점프 날개, 궤도 구슬). 분신은 내 사격과 같은 발 수, 차지샷도 멀티샷 수만큼, 두꺼비는 절벽을 피함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="46" customHeight="1" s="37">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>0.4.3 변경</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>기본 필살기 너프(35+3/단계, 보스 120). 보스 외 적 체력 +6 (슬라임·마법사·두꺼비 26, 늑대 36, 박쥐 16, 작은 슬라임 16). 대시 칸 카드가 공중 대시 횟수도 늘림. 분신 최대 3마리(한 줄로 따라옴). 상점 뽑기 가격 +25씩, 카드 강화 칸 추가. 영웅·전설 확률 크게 낮춤.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>0.4.4 변경</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>전설 확률 3 / 5 / 8% (일반을 그만큼 낮춤). 상점 뽑기 가격은 100코인에서 더 오르지 않음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>0.4.5 변경</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>웨이브 공이 바닥에 바로 닿아 사라지던 문제 수정. 등급 확률을 스테이지 1 일반 50% 기준으로 재조정. 상점 강화 화면을 목록형으로 다시 만듦.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>0.4.6 변경</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>그림자 분신은 0.8초마다 플레이어와 같은 공격을 쏜다(내 사격을 따라 하지 않음). 상점 뽑기 가격은 상한 없이 그 판에서 뽑을 때마다 +25, 다음 상점에도 이어진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>0.4.7 변경</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>사거리 계산을 한 곳으로(산탄 55%는 판 내내 유지, 능력치 패널 RANGE 가 실제 값). AIR JUMP 를 DOUBLE JUMP 로 이름 변경. 전설 이동 카드 그림자 날개(비행) 추가.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="37" min="1" max="1"/>
+    <col width="22" customWidth="1" style="37" min="2" max="2"/>
+    <col width="90" customWidth="1" style="37" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>스테이지 1·2 구성 (0.4.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>열 = 타일 x (1칸 32px), 바닥 윗면 = 15행. 배치 코드는 Source/Private/world/StageBuilder.cpp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>요소</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>동작</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>보상 / 규칙</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>매복 결투장</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>들어오면 양 끝 열에 마법 벽이 생기고 카메라가 결투장 화면에 묶인다. 다음 웨이브 자리에 0.8~1초 동안 소환 마법진(정예는 금빛)이 돌고 적이 나온다. 0.4.1 긴장감: 화면 가장자리가 붉게 맥박치고, HUD 에 WAVE n/m 과 제한 시간 바(스테이지 1은 20초, 2는 16초). 마지막 5초는 빨갛게 깜빡이며 째깍 소리, 시간이 다 되면 남은 적이 있어도 다음 웨이브가 증원으로 나온다 (마지막 웨이브는 제한 없음)</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>웨이브를 모두 잡으면 벽이 열리고 가운데에 보물상자가 떨어진다. 결투장 박쥐는 7~8행 (가운데 발판에 올라서면 맞는 높이). 제한 시간 안에 웨이브를 정리하면 남은 3초마다 코인 1 (FAST +n)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>점프 버섯</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>바닥에 박힌 분홍 버섯. 밟고 지나가기만 해도 약 9칸 높이로 튀어 오르고 공중 점프·공중 대시가 다시 찬다.</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>절벽·가시밭을 넘거나 높은 길(숨은 상자)로 올라갈 때 쓴다</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="inlineStr">
+        <is>
+          <t>정예 적</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>금빛 기운과 체력 바, 체력 3배 (최소 +40). 스킬을 쓰기 전 머리 위에 빨간 "!" 로 0.5초 예고</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>경험치 4배, 코인 12, 하트 50%, 점수 500. 스킬(0.4.1): 슬라임 = 3초마다 플레이어 쪽으로 크게 뛰어들기, 쓰러지면 작은 슬라임 3 / 늑대 = 가까우면 빠르게 덮치기 / 마법사 = 부채꼴 3발 / 박쥐 = 3초마다 급강하 / 두꺼비 = 착지할 때 좌우 짧은 충격파</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="inlineStr">
+        <is>
+          <t>보물상자</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>아래 지면으로 떨어져 앉아 반짝인다. 닿으면 열린다.</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>코인 15 + 보너스 카드 1장 + 점수 300</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>깃발</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>기둥 위로 뛰어넘어도 클리어되도록 판정을 화면 위끝까지 넓힘</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>그림자 두꺼비 (0.4.1 새 적)</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>웅크렸다가 플레이어 쪽으로 크게 뛰어든다 (멀면 제자리에서 작게). 체력 26+10x스테이지, 경험치 3. 0.4.2: 뛰기 전에 떨어질 자리를 보고 구덩이면 덜 뛰거나 제자리에서 뛴다</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>스테이지 1·2 의 길과 결투장 웨이브에 섞여 나온다. 정예는 착지 충격파</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>스테이지</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>구간 (열)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>1 MISTY FIELDS (160칸)</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>0~25</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>슬라임 2, 첫 점프 버섯(6열) 위 발판의 코인, 구덩이</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="inlineStr"/>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>26~55 결투장 1</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>W1 슬라임 3 / W2 늑대 2 + 발판 위 슬라임</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="inlineStr"/>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>56~99</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>버섯으로 넘는 절벽(57열), 발판 위 마법사, 박쥐, 정예 늑대(81열), 버섯(86열) 위 높은 길의 숨은 상자(91열), 하트</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="inlineStr"/>
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>100~129 결투장 2</t>
+        </is>
+      </c>
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>W1 늑대 2 + 박쥐 2 / W2 마법사 2 + 슬라임 2 / W3 정예 늑대 + 슬라임 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="38" t="inlineStr"/>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>130~159</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="inlineStr">
+        <is>
+          <t>슬라임, 박쥐, 계단, 깃발(155열)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>2 WHISPERING CAVE (180칸)</t>
+        </is>
+      </c>
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>0~39</t>
+        </is>
+      </c>
+      <c r="C18" s="38" t="inlineStr">
+        <is>
+          <t>천장. 입구 적, 무너지는 다리, 버섯(28열)으로 넘는 가시밭</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="inlineStr"/>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>40~69 결투장 1</t>
+        </is>
+      </c>
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>W1 슬라임 3 + 박쥐 / W2 마법사 2 + 늑대 2 / W3 정예 마법사 + 박쥐 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="38" t="inlineStr"/>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>70~113</t>
+        </is>
+      </c>
+      <c r="C20" s="38" t="inlineStr">
+        <is>
+          <t>무너지는 다리, 버섯(78열) + 가시밭, 정예 슬라임(89열), 버섯(95열) 위 천장 아래 숨은 상자(99열), 하트</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="38" t="inlineStr"/>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>114~143 결투장 2</t>
+        </is>
+      </c>
+      <c r="C21" s="38" t="inlineStr">
+        <is>
+          <t>W1 늑대 3 / W2 마법사 2 + 박쥐 2 + 슬라임 / W3 정예 늑대 + 정예 마법사 + 박쥐</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="inlineStr"/>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>144~179</t>
+        </is>
+      </c>
+      <c r="C22" s="38" t="inlineStr">
+        <is>
+          <t>버섯(148열) + 가시밭, 적, 계단, 깃발(176열)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>검증 봇 (bot=1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>목표 재탐색</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>30프레임마다 우선순위대로 목표를 다시 고른다: 결투장 적 &gt; 500px 안의 닫힌 보물상자 &gt; 지나쳐 버린 깃발 &gt; 전진</t>
+        </is>
+      </c>
+      <c r="C25" s="42" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>결투장</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>① 결투장 적만 목표 (같은 높이 우선) ② 위면 뛰어올라 발판, 아래면 발판 끝으로 내려감 ③ 120~260px 거리, 목표 쪽을 봄 ④ 계속 공격</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B24:C24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1022,7 +1476,7 @@
     <row r="2" ht="42" customHeight="1" s="37">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>보스 체력 300 고정. 체력 66% / 33% 아래로 내려가면 단계가 오르고(RAGE / FURY 배너) 카드를 1장씩 고른다. 단계마다 아래 목록에서 무작위로 고르며, 공격 사이 쉬는 시간은 60/48/36프레임. 수치는 "1단계 / 2단계 / 3단계" 순 (Source/Private/data/BossTuning.cpp). 60프레임 = 1초.</t>
+          <t>보스 체력 3000 고정 (0.4.2: 피해 10단위. 예전 단위 600 을 목표로, 공격력 3단계 빌드에서 같은 타수가 되게). 체력 66% / 33% 아래로 내려가면 단계가 오르고(RAGE / FURY 배너) 카드를 1장씩 고른다. 단계마다 아래 목록에서 무작위로 고르며, 공격 사이 쉬는 시간은 60/48/36프레임. 수치는 "1단계 / 2단계 / 3단계" 순 (Source/Private/data/BossTuning.cpp). 60프레임 = 1초.</t>
         </is>
       </c>
     </row>
@@ -1220,12 +1674,12 @@
       </c>
       <c r="H6" s="38" t="inlineStr">
         <is>
-          <t>양쪽에서 박쥐 2마리를 부름 (이미 4마리 이상이면 생략)</t>
+          <t>양쪽에서 박쥐 2마리를 부름 (이미 4마리 이상이면 생략). 0.4.1: 박쥐가 순찰하지 않고 플레이어를 향해 천천히(1.7px/프레임) 날아옴</t>
         </is>
       </c>
       <c r="I6" s="38" t="inlineStr">
         <is>
-          <t>박쥐를 먼저 정리</t>
+          <t>박쥐를 먼저 정리. 다가오는 길목에 공을 깔아 둔다</t>
         </is>
       </c>
       <c r="J6" s="38" t="inlineStr">
@@ -2423,13 +2877,13 @@
         </is>
       </c>
       <c r="F4" s="19" t="n">
-        <v>0.44</v>
+        <v>0.5</v>
       </c>
       <c r="G4" s="19" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="H4" s="19" t="n">
         <v>0.36</v>
-      </c>
-      <c r="H4" s="19" t="n">
-        <v>0.28</v>
       </c>
       <c r="I4" s="39" t="n">
         <v>-0.05</v>
@@ -2458,13 +2912,13 @@
         </is>
       </c>
       <c r="F5" s="19" t="n">
-        <v>0.32</v>
+        <v>0.36</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="I5" s="39" t="n">
         <v>0.02</v>
@@ -2493,13 +2947,13 @@
         </is>
       </c>
       <c r="F6" s="19" t="n">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>0.22</v>
+        <v>0.13</v>
       </c>
       <c r="H6" s="19" t="n">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="I6" s="39" t="n">
         <v>0.02</v>
@@ -2528,13 +2982,13 @@
         </is>
       </c>
       <c r="F7" s="19" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="G7" s="19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="19" t="n">
         <v>0.08</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>0.1</v>
       </c>
       <c r="I7" s="39" t="n">
         <v>0.01</v>
@@ -2580,7 +3034,7 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>· 사용자 요청: 전설 확률을 스테이지 1/2/3에서 6% / 8% / 10%로. 나머지 등급도 같이 올려서 일반이 절반 아래가 되게 했다 (게임이 늘어지지 않도록).</t>
+          <t>· 0.4.5: 스테이지 1 일반 50% 기준으로 다시 맞춤. 일반 50/43/36%, 희귀 36/39/41%, 영웅 11/13/15%, 전설 3/5/8%</t>
         </is>
       </c>
     </row>
@@ -2630,7 +3084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" style="37" min="1" max="1"/>
@@ -2754,12 +3208,12 @@
       </c>
       <c r="G2" s="38" t="inlineStr">
         <is>
-          <t>섀도우볼 피해 증가 (공이 커지는 연출 유지)</t>
+          <t>섀도우볼 피해 증가 (공이 커지는 연출 유지). 0.4.2: 피해 10단위 (기본 10, 단계마다 +3, 최대 25)</t>
         </is>
       </c>
       <c r="H2" s="26" t="inlineStr">
         <is>
-          <t>피해 +1</t>
+          <t>피해 +3</t>
         </is>
       </c>
       <c r="I2" s="27" t="n">
@@ -2783,7 +3237,7 @@
       </c>
       <c r="N2" s="38" t="inlineStr">
         <is>
-          <t>기존 공격력 업그레이드(최대 4)를 5로. 밸런스: 너무 안 나와서 일반 -&gt; 희귀, 비중 4배. 0.3.1: 비중 4일 때 레벨업 화면 한 번에 나올 확률이 약 20%(희귀 칸의 4/19)라 너무 자주 보여서 비중 2로 (약 11%)</t>
+          <t>기존 공격력 업그레이드(최대 4)를 5로. 0.4.2: 한 장에 피해가 두 배가 되던 1 단위를 10 단위로 바꾸고, 뽑힐 비중도 같은 등급 카드와 같게(1) — 비중 4·2 모두 너무 자주 나왔다</t>
         </is>
       </c>
     </row>
@@ -2909,7 +3363,11 @@
           <t>하</t>
         </is>
       </c>
-      <c r="N4" s="38" t="n"/>
+      <c r="N4" s="38" t="inlineStr">
+        <is>
+          <t>0.4.7: 실제 사거리 = 속도 x 수명(기본 36 + 공격력 단계마다 3, 사거리 +20%/단계) x 튕김 1.6 x 산탄 0.55 x 레이저 2.6배 속도. 능력치 패널 RANGE 가 이 값</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -3383,7 +3841,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>영웅</t>
+          <t>희귀</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -3427,7 +3885,7 @@
       </c>
       <c r="N12" s="38" t="inlineStr">
         <is>
-          <t>타일 충돌 시 반사, 뜬 발판은 통과. 0.2.3 재설계: 벽에서만 튕겨서 쓸모가 적었음 → 적에게도 튕김. 3/5번일 때 보스 피해가 약 4배여서 2/3번으로 조정</t>
+          <t>타일 충돌 시 반사, 뜬 발판은 통과. 0.2.3 재설계: 벽에서만 튕겨서 쓸모가 적었음 → 적에게도 튕김. 3/5번일 때 보스 피해가 약 4배여서 2/3번으로 조정 / 0.4.2: 영웅 -&gt; 희귀</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3973,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>영웅</t>
+          <t>희귀</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -3559,7 +4017,7 @@
       </c>
       <c r="N14" s="38" t="inlineStr">
         <is>
-          <t>밸런스: +25% 는 기본 피해 1에서 반올림되어 효과가 없었음 -&gt; 2초간 2배. 보스에게 2배가 계속 이어지지 않도록 대상별 15초 쿨타임</t>
+          <t>밸런스: +25% 는 기본 피해 1에서 반올림되어 효과가 없었음 -&gt; 2초간 2배. 보스에게 2배가 계속 이어지지 않도록 대상별 15초 쿨타임 / 0.4.2: 영웅 -&gt; 희귀</t>
         </is>
       </c>
     </row>
@@ -3581,7 +4039,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>전설</t>
+          <t>영웅</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -3596,12 +4054,12 @@
       </c>
       <c r="G15" s="38" t="inlineStr">
         <is>
-          <t>섀도우볼이 가장 가까운 적을 향해 휘어서 날아감. 대신 공격력 -1 (최소 1)</t>
+          <t>섀도우볼이 가장 가까운 적을 향해 휘어서 날아감. 대신 피해 -3 (최소 7)</t>
         </is>
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
-          <t>유도 / 공격력 -1</t>
+          <t>유도 / 피해 -3</t>
         </is>
       </c>
       <c r="I15" s="27" t="n">
@@ -3625,7 +4083,7 @@
       </c>
       <c r="N15" s="38" t="inlineStr">
         <is>
-          <t>사용자: 전설 카드. 밸런스: 맞히기 쉬운 대신 공격력 -1 (최소 1)</t>
+          <t>사용자: 전설 카드였으나 0.4.2 새 카드(혈사포 등)가 늘어 영웅으로. 맞히기 쉬운 대신 피해 -3</t>
         </is>
       </c>
     </row>
@@ -3713,7 +4171,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>전설</t>
+          <t>영웅</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -3757,7 +4215,7 @@
       </c>
       <c r="N17" s="38" t="inlineStr">
         <is>
-          <t>누르고 있는 동안 연사는 멈춤. 단계마다 빛 색(보라→하늘→분홍→금)과 머리 위 점으로 표시. 0.2.3: 1초 3배 고정은 보스전에서 손해라 단계식으로</t>
+          <t>누르고 있는 동안 연사는 멈춤. 단계마다 빛 색(보라→하늘→분홍→금)과 머리 위 점으로 표시. 0.2.3: 1초 3배 고정은 보스전에서 손해라 단계식으로 / 0.4.2: 멀티샷이 있으면 차지 공도 같은 수만큼 부채꼴로. 혈사포와 함께 나오지 않음. 전설 -&gt; 영웅</t>
         </is>
       </c>
     </row>
@@ -4050,12 +4508,12 @@
       </c>
       <c r="G22" s="38" t="inlineStr">
         <is>
-          <t>몸통으로 부딪힌 적에게 피해 3</t>
+          <t>부딪힌 적에게 피해 30</t>
         </is>
       </c>
       <c r="H22" s="26" t="inlineStr">
         <is>
-          <t>반격 3</t>
+          <t>반격 30</t>
         </is>
       </c>
       <c r="I22" s="27" t="n">
@@ -4339,12 +4797,12 @@
       </c>
       <c r="B27" s="38" t="inlineStr">
         <is>
-          <t>다단 점프</t>
+          <t>더블 점프</t>
         </is>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
-          <t>AIR JUMP</t>
+          <t>DOUBLE JUMP</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -4393,7 +4851,7 @@
       </c>
       <c r="N27" s="38" t="inlineStr">
         <is>
-          <t>기존 이단 점프(최대 1)를 2로</t>
+          <t>기존 이단 점프(최대 1)를 2로 0.4.2: 등 뒤에 작은 박쥐 날개 (단계마다 한 쌍) / 0.4.7: 게임 표기 AIR JUMP -&gt; DOUBLE JUMP (더블 점프 카드가 없는 줄 알아서)</t>
         </is>
       </c>
     </row>
@@ -4624,7 +5082,7 @@
       </c>
       <c r="G31" s="38" t="inlineStr">
         <is>
-          <t>대시 칸 +1 (연속으로 대시 가능, HUD에 칸 표시)</t>
+          <t>대시 칸 +1 (연속으로 대시 가능, HUD에 칸 표시). 공중 대시 횟수도 +1</t>
         </is>
       </c>
       <c r="H31" s="26" t="inlineStr">
@@ -4653,7 +5111,7 @@
       </c>
       <c r="N31" s="38" t="inlineStr">
         <is>
-          <t>사용자: 대시 가능 칸 + 횟수 증가. 기본 1칸 → 최대 3칸. 중첩 가능한 특수 능력</t>
+          <t>사용자: 대시 가능 칸 + 횟수 증가. 기본 1칸 → 최대 3칸. 중첩 가능한 특수 능력 / 0.4.3: 공중에서는 연속 대시가 안 되던 문제 -&gt; 공중 대시 횟수 = 1 + 공중 대시 + 대시 칸</t>
         </is>
       </c>
     </row>
@@ -5857,21 +6315,21 @@
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>특수</t>
+          <t>특수(중첩)</t>
         </is>
       </c>
       <c r="G50" s="38" t="inlineStr">
         <is>
-          <t>작은 겐가 분신이 따라다니며 0.8초마다 가장 가까운 적에게 자동 사격 (내 공의 특수 능력도 같이 적용)</t>
+          <t>작은 겐가 분신이 플레이어 뒤로 한 줄로 따라다니며 0.8초마다 플레이어와 같은 공격(같은 발 수, 같은 공 능력, 크기 70%·피해 50%)을 가장 가까운 적에게 쏜다. 최대 3마리</t>
         </is>
       </c>
       <c r="H50" s="26" t="inlineStr">
         <is>
-          <t>분신 1</t>
+          <t>분신 +1</t>
         </is>
       </c>
       <c r="I50" s="27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J50" s="38" t="n"/>
       <c r="K50" s="38" t="inlineStr">
@@ -5891,13 +6349,739 @@
       </c>
       <c r="N50" s="38" t="inlineStr">
         <is>
-          <t>도트 스프라이트 1종 추가 필요. 0.3.1: 스테이지 중에 얻으면 다음 스테이지가 아니라 바로 나오도록 수정</t>
+          <t>0.4.6: 내 사격에 맞춰 쏘던 것(0.4.2)을 다시 0.8초 주기로. 여러 마리면 쏘는 때를 0.27초씩 엇갈림. 0.4.3: 최대 3마리</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="27" customHeight="1" s="37">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>A17</t>
+        </is>
+      </c>
+      <c r="B51" s="38" t="inlineStr">
+        <is>
+          <t>혈사포</t>
+        </is>
+      </c>
+      <c r="C51" s="38" t="inlineStr">
+        <is>
+          <t>BRIMSTONE</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>전설</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G51" s="38" t="inlineStr">
+        <is>
+          <t>보통 공 대신 Z 를 0.75초 모았다가 떼면 화면 끝까지 굵은 핏빛 광선 0.5초. 모든 적 관통, 3프레임마다 공격력 x0.6 (약 6배)</t>
+        </is>
+      </c>
+      <c r="H51" s="26" t="inlineStr">
+        <is>
+          <t>광선</t>
+        </is>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" s="38" t="inlineStr">
+        <is>
+          <t>차지샷·레이저 없음</t>
+        </is>
+      </c>
+      <c r="K51" s="38" t="inlineStr">
+        <is>
+          <t>핏빛 광선 + 뿔</t>
+        </is>
+      </c>
+      <c r="L51" s="38" t="inlineStr">
+        <is>
+          <t>사용자</t>
+        </is>
+      </c>
+      <c r="M51" s="10" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="N51" s="38" t="inlineStr">
+        <is>
+          <t>아이작의 혈사포. 멀티샷 1발마다 광선 10px 굵게. 얻으면 머리에 빨간 뿔</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="27" customHeight="1" s="37">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="B52" s="38" t="inlineStr">
+        <is>
+          <t>레이저</t>
+        </is>
+      </c>
+      <c r="C52" s="38" t="inlineStr">
+        <is>
+          <t>LASER</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>영웅</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G52" s="38" t="inlineStr">
+        <is>
+          <t>공이 2.6배 빠른 가는 레이저가 되어 모든 적을 관통. 피해 70%</t>
+        </is>
+      </c>
+      <c r="H52" s="26" t="inlineStr">
+        <is>
+          <t>레이저</t>
+        </is>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" s="38" t="inlineStr">
+        <is>
+          <t>혈사포 없음</t>
+        </is>
+      </c>
+      <c r="K52" s="38" t="inlineStr">
+        <is>
+          <t>분홍 빛줄기</t>
+        </is>
+      </c>
+      <c r="L52" s="38" t="inlineStr">
+        <is>
+          <t>사용자</t>
+        </is>
+      </c>
+      <c r="M52" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N52" s="38" t="inlineStr">
+        <is>
+          <t>공 모양 변경</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="27" customHeight="1" s="37">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>A19</t>
+        </is>
+      </c>
+      <c r="B53" s="38" t="inlineStr">
+        <is>
+          <t>부메랑</t>
+        </is>
+      </c>
+      <c r="C53" s="38" t="inlineStr">
+        <is>
+          <t>BOOMERANG</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G53" s="38" t="inlineStr">
+        <is>
+          <t>사거리 절반에서 돌아서 플레이어에게 돌아오며 다시 맞힘</t>
+        </is>
+      </c>
+      <c r="H53" s="26" t="inlineStr">
+        <is>
+          <t>되돌아옴</t>
+        </is>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="38" t="n"/>
+      <c r="K53" s="38" t="inlineStr">
+        <is>
+          <t>휘어진 화살표</t>
+        </is>
+      </c>
+      <c r="L53" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M53" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N53" s="38" t="inlineStr">
+        <is>
+          <t>공 모양 변경</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="27" customHeight="1" s="37">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>A20</t>
+        </is>
+      </c>
+      <c r="B54" s="38" t="inlineStr">
+        <is>
+          <t>웨이브</t>
+        </is>
+      </c>
+      <c r="C54" s="38" t="inlineStr">
+        <is>
+          <t>WAVE SHOT</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G54" s="38" t="inlineStr">
+        <is>
+          <t>공이 진행 방향 옆으로 사인파(진폭 16px)처럼 출렁임. 처음에는 위로 출렁이고, 벽·바닥 충돌은 출렁임을 뺀 중심선으로 판단</t>
+        </is>
+      </c>
+      <c r="H54" s="26" t="inlineStr">
+        <is>
+          <t>출렁임</t>
+        </is>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J54" s="38" t="n"/>
+      <c r="K54" s="38" t="inlineStr">
+        <is>
+          <t>물결</t>
+        </is>
+      </c>
+      <c r="L54" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M54" s="10" t="inlineStr">
+        <is>
+          <t>하</t>
+        </is>
+      </c>
+      <c r="N54" s="38" t="inlineStr">
+        <is>
+          <t>공 모양 변경. 0.4.5: 바닥 가까이서 쏘면 출렁임 때문에 바로 땅에 닿아 사라지던 문제 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="27" customHeight="1" s="37">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>A21</t>
+        </is>
+      </c>
+      <c r="B55" s="38" t="inlineStr">
+        <is>
+          <t>산탄</t>
+        </is>
+      </c>
+      <c r="C55" s="38" t="inlineStr">
+        <is>
+          <t>SCATTER</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G55" s="38" t="inlineStr">
+        <is>
+          <t>공 +2발을 넓은 부채꼴로. 사거리 55%, 한 발 피해 80%</t>
+        </is>
+      </c>
+      <c r="H55" s="26" t="inlineStr">
+        <is>
+          <t>+2발</t>
+        </is>
+      </c>
+      <c r="I55" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J55" s="38" t="n"/>
+      <c r="K55" s="38" t="inlineStr">
+        <is>
+          <t>퍼지는 점</t>
+        </is>
+      </c>
+      <c r="L55" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M55" s="10" t="inlineStr">
+        <is>
+          <t>하</t>
+        </is>
+      </c>
+      <c r="N55" s="38" t="inlineStr">
+        <is>
+          <t>근접 메타</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="27" customHeight="1" s="37">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="B56" s="38" t="inlineStr">
+        <is>
+          <t>무거운 공</t>
+        </is>
+      </c>
+      <c r="C56" s="38" t="inlineStr">
+        <is>
+          <t>HEAVY SHOT</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="E56" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G56" s="38" t="inlineStr">
+        <is>
+          <t>공 크기 1.45배, 피해 +40%, 연사 25% 느림</t>
+        </is>
+      </c>
+      <c r="H56" s="26" t="inlineStr">
+        <is>
+          <t>크고 느림</t>
+        </is>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J56" s="38" t="n"/>
+      <c r="K56" s="38" t="inlineStr">
+        <is>
+          <t>큰 공</t>
+        </is>
+      </c>
+      <c r="L56" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M56" s="10" t="inlineStr">
+        <is>
+          <t>하</t>
+        </is>
+      </c>
+      <c r="N56" s="38" t="n"/>
+    </row>
+    <row r="57" ht="27" customHeight="1" s="37">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="B57" s="38" t="inlineStr">
+        <is>
+          <t>독</t>
+        </is>
+      </c>
+      <c r="C57" s="38" t="inlineStr">
+        <is>
+          <t>POISON</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F57" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G57" s="38" t="inlineStr">
+        <is>
+          <t>맞은 적이 3초 동안 0.5초마다 그 피해의 25% (약 1.5배 더). 보스도 걸림</t>
+        </is>
+      </c>
+      <c r="H57" s="26" t="inlineStr">
+        <is>
+          <t>지속 피해</t>
+        </is>
+      </c>
+      <c r="I57" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J57" s="38" t="n"/>
+      <c r="K57" s="38" t="inlineStr">
+        <is>
+          <t>초록 방울</t>
+        </is>
+      </c>
+      <c r="L57" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M57" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N57" s="38" t="inlineStr">
+        <is>
+          <t>머리 위 초록 방울 표시</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="27" customHeight="1" s="37">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="B58" s="38" t="inlineStr">
+        <is>
+          <t>냉기</t>
+        </is>
+      </c>
+      <c r="C58" s="38" t="inlineStr">
+        <is>
+          <t>FROST</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G58" s="38" t="inlineStr">
+        <is>
+          <t>맞은 적이 2초 동안 이동 속도 절반. 보스는 느려지지 않음</t>
+        </is>
+      </c>
+      <c r="H58" s="26" t="inlineStr">
+        <is>
+          <t>느려짐</t>
+        </is>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J58" s="38" t="n"/>
+      <c r="K58" s="38" t="inlineStr">
+        <is>
+          <t>눈송이</t>
+        </is>
+      </c>
+      <c r="L58" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M58" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N58" s="38" t="inlineStr">
+        <is>
+          <t>머리 위 눈송이 표시</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="27" customHeight="1" s="37">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>A25</t>
+        </is>
+      </c>
+      <c r="B59" s="38" t="inlineStr">
+        <is>
+          <t>연쇄 번개</t>
+        </is>
+      </c>
+      <c r="C59" s="38" t="inlineStr">
+        <is>
+          <t>CHAIN BOLT</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>영웅</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F59" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G59" s="38" t="inlineStr">
+        <is>
+          <t>맞힐 때마다 170px 안의 가장 가까운 다른 적에게 번개 50%</t>
+        </is>
+      </c>
+      <c r="H59" s="26" t="inlineStr">
+        <is>
+          <t>연쇄 1</t>
+        </is>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J59" s="38" t="n"/>
+      <c r="K59" s="38" t="inlineStr">
+        <is>
+          <t>번개</t>
+        </is>
+      </c>
+      <c r="L59" s="38" t="inlineStr">
+        <is>
+          <t>기획 추가</t>
+        </is>
+      </c>
+      <c r="M59" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N59" s="38" t="n"/>
+    </row>
+    <row r="60" ht="27" customHeight="1" s="37">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
+      </c>
+      <c r="B60" s="38" t="inlineStr">
+        <is>
+          <t>그림자 궤도</t>
+        </is>
+      </c>
+      <c r="C60" s="38" t="inlineStr">
+        <is>
+          <t>SHADOW ORBIT</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>영웅</t>
+        </is>
+      </c>
+      <c r="E60" s="10" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
+          <t>특수(중첩)</t>
+        </is>
+      </c>
+      <c r="G60" s="38" t="inlineStr">
+        <is>
+          <t>몸 주위를 도는 구슬 2개(2단계 4개). 닿은 적에게 공격력 x0.6, 적 탄환을 막음</t>
+        </is>
+      </c>
+      <c r="H60" s="26" t="inlineStr">
+        <is>
+          <t>구슬 +2</t>
+        </is>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J60" s="38" t="n"/>
+      <c r="K60" s="38" t="inlineStr">
+        <is>
+          <t>도는 구슬</t>
+        </is>
+      </c>
+      <c r="L60" s="38" t="inlineStr">
+        <is>
+          <t>사용자</t>
+        </is>
+      </c>
+      <c r="M60" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N60" s="38" t="inlineStr">
+        <is>
+          <t>따라다니는 친구처럼 겉모습이 바뀌는 카드</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>M06</t>
+        </is>
+      </c>
+      <c r="B61" s="38" t="inlineStr">
+        <is>
+          <t>그림자 날개</t>
+        </is>
+      </c>
+      <c r="C61" s="38" t="inlineStr">
+        <is>
+          <t>SHADOW WINGS</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>전설</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>이동</t>
+        </is>
+      </c>
+      <c r="F61" s="10" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="G61" s="38" t="inlineStr">
+        <is>
+          <t>등 뒤에 큰 날개가 돋고, 공중에서 점프를 누르고 있으면 위로 난다. 비행 2.5초(몸 아래 바), 땅에 있으면 다시 참. 다 쓰면 천천히 활공</t>
+        </is>
+      </c>
+      <c r="H61" s="26" t="inlineStr">
+        <is>
+          <t>비행 2.5초</t>
+        </is>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J61" s="38" t="n"/>
+      <c r="K61" s="38" t="inlineStr">
+        <is>
+          <t>큰 박쥐 날개</t>
+        </is>
+      </c>
+      <c r="L61" s="38" t="inlineStr">
+        <is>
+          <t>사용자</t>
+        </is>
+      </c>
+      <c r="M61" s="10" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="N61" s="38" t="inlineStr">
+        <is>
+          <t>0.4.7 추가. 화면 맨 위 근처로는 못 올라감. 겉모습이 바뀌는 카드</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N50"/>
-  <conditionalFormatting sqref="D2:D50">
+  <autoFilter ref="A1:N61"/>
+  <conditionalFormatting sqref="D2:D60">
     <cfRule type="expression" priority="1" dxfId="7">
       <formula>$D2="일반"</formula>
     </cfRule>
@@ -5911,7 +7095,7 @@
       <formula>$D2="전설"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F50">
+  <conditionalFormatting sqref="F2:F60">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>$F2="능력치"</formula>
     </cfRule>
@@ -5950,7 +7134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="30" customWidth="1" style="37" min="1" max="1"/>
@@ -6326,6 +7510,125 @@
       <c r="C25" s="38" t="inlineStr">
         <is>
           <t>공 하나당 분열 1번 (적이든 벽이든 먼저 닿은 곳)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>혈사포 + 차지샷 / 레이저</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>함께 나오지 않음 (혈사포가 있으면 둘은 제시 목록에서 빠지고, 반대도 같다)</t>
+        </is>
+      </c>
+      <c r="C26" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>혈사포 + 멀티샷</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>광선이 1발마다 10px 굵어짐</t>
+        </is>
+      </c>
+      <c r="C27" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>혈사포 + 저주/독/냉기/치명타</t>
+        </is>
+      </c>
+      <c r="B28" s="38" t="inlineStr">
+        <is>
+          <t>광선 한 번 한 번에 모두 적용</t>
+        </is>
+      </c>
+      <c r="C28" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="inlineStr">
+        <is>
+          <t>차지샷 + 멀티샷 (0.4.2)</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>차지 공도 멀티샷 수만큼 부채꼴로</t>
+        </is>
+      </c>
+      <c r="C29" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>산탄 + 멀티샷</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>발 수가 더해짐 (예: 멀티샷 2 + 산탄 = 5발)</t>
+        </is>
+      </c>
+      <c r="C30" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>분신 + 모든 사격</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>0.8초마다 내 공격과 같은 발 수, 같은 공 능력 (피해 50%)</t>
+        </is>
+      </c>
+      <c r="C31" s="38" t="inlineStr">
+        <is>
+          <t>쏠 적이 없으면 쏘지 않는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>부메랑 + 관통/튕김</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>돌아오는 길에 이미 맞힌 적도 다시 맞힘</t>
+        </is>
+      </c>
+      <c r="C32" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6431,14 +7734,14 @@
       </c>
       <c r="E4" s="38" t="inlineStr">
         <is>
-          <t>화면 전체에 충격파 한 번. 화면 안의 적 전부에게 피해 (지금 필살기 그대로)</t>
+          <t>화면 전체에 충격파 한 번. 화면 안의 적 전부에게 피해. 0.4.3: 광역이라 너프 (일반 35 + 공격력 단계마다 3, 보스 120). 피해 10단위</t>
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="G4" s="27" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="H4" s="27" t="n">
         <v>0</v>
@@ -7199,7 +8502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" style="37" min="1" max="1"/>
@@ -7226,7 +8529,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>확정: 1회 50코인 고정. 오르는 가격은 0 (나중에 바꾸고 싶으면 B4만 고치면 된다)</t>
+          <t>0.4.6: 첫 뽑기 50코인, 그 판에서 뽑을 때마다 +25, 상한 없음. 다음 상점에도 이어진다 (스테이지 1 뒤 상점에서 75까지 뽑았으면 스테이지 2 뒤 상점은 100부터)</t>
         </is>
       </c>
     </row>
@@ -7237,7 +8540,7 @@
         </is>
       </c>
       <c r="B4" s="33" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -7248,7 +8551,7 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>50코인 고정 (확정)</t>
+          <t>50 + 25 x (이번 판에서 상점에서 뽑은 횟수)</t>
         </is>
       </c>
     </row>
@@ -7675,21 +8978,104 @@
       <c r="G34" s="41" t="n"/>
       <c r="H34" s="42" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>카드 강화 (0.4.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>위치</t>
+        </is>
+      </c>
+      <c r="B37" s="38" t="inlineStr">
+        <is>
+          <t>오른쪽 가운데 칸 (뽑기 아래, 다음 스테이지 위). 예전 안내 글 자리에 만들고 출발 칸과 자리를 바꿈</t>
+        </is>
+      </c>
+      <c r="C37" s="41" t="n"/>
+      <c r="D37" s="41" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="41" t="n"/>
+      <c r="G37" s="41" t="n"/>
+      <c r="H37" s="42" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="inlineStr">
+        <is>
+          <t>대상</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>얻은 카드 중 같은 카드를 또 얻으면 단계가 오르는 것(능력치, 특수(중첩))이고 아직 최대 단계가 아닌 것</t>
+        </is>
+      </c>
+      <c r="C38" s="41" t="n"/>
+      <c r="D38" s="41" t="n"/>
+      <c r="E38" s="41" t="n"/>
+      <c r="F38" s="41" t="n"/>
+      <c r="G38" s="41" t="n"/>
+      <c r="H38" s="42" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>등급 기본값 + 지금 단계 x 20. 기본값: 일반 60 / 희귀 90 / 영웅 140 / 전설 200 (뽑기 첫 가격 50 보다 비싸게)</t>
+        </is>
+      </c>
+      <c r="C39" s="41" t="n"/>
+      <c r="D39" s="41" t="n"/>
+      <c r="E39" s="41" t="n"/>
+      <c r="F39" s="41" t="n"/>
+      <c r="G39" s="41" t="n"/>
+      <c r="H39" s="42" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>조작</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>0.4.5 목록형으로 다시: 강화 칸에서 Z -&gt; 올릴 수 있는 카드가 한 줄씩(아이콘, 이름, 등급, 단계 칸에서 오를 칸은 금색, LV 2 &gt; 3, 가격). ↑ ↓ 로 고르고 Z 로 올림, Esc 로 돌아감. 위에 가진 코인과 "무엇을 하는 화면인지" 설명, 아래에 고른 카드의 자세한 설명과 "Z 를 누르면 몇 코인" 안내. 코인이 모자라면 가격과 안내가 빨갛다</t>
+        </is>
+      </c>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="41" t="n"/>
+      <c r="G40" s="41" t="n"/>
+      <c r="H40" s="42" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="18">
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B32:H32"/>
     <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B26:H26"/>
     <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B40:H40"/>
     <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B39:H39"/>
     <mergeCell ref="B34:H34"/>
     <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B38:H38"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B19:H19"/>
     <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B37:H37"/>
     <mergeCell ref="B28:H28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>